<commit_message>
update: mise à jour notebooks SVM + figures + présentation
- analyse_SVM.ipynb : sections 8c, 9b, 12 finalisées (zones validité, arbres RF, isosurfaces)
- analyse_kfold.ipynb : comparaison K-Fold vs LOOCV mise à jour
- Figures régénérées : visualisation 3D, zones validité, importance features, optimisation RF
- presentation_B430.html : mise à jour présentation
- CLAUDE.md : documentation architecture notebook complétée
- bilan SVM.xlsx : données mises à jour

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bilan SVM.xlsx
+++ b/bilan SVM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d542b0eedbde6f23/Documents/dèv/projet_SVM_fiabila/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{4E7CE648-3759-41E5-8840-F16BD7962D81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A5EF104-4DAA-4284-BD94-DCE3A1340CB2}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{87BAAAC3-05E7-449E-A9A6-4FAD689F0B13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5DC5BE76-6E9B-4EF6-A34E-08006DFF6504}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -71,7 +71,7 @@
     <t>MOYENNE</t>
   </si>
   <si>
-    <t>ℹ  N/D = donnée non disponible (exclue de la moyenne). Les 20 lots bons produit et 8 lots mauvais produit sont issus de Sheet1.</t>
+    <t>ℹ  N/D = donnée non disponible (exclue de la moyenne). Les 21 lots bons produit et 13 lots mauvais produit sont issus de Sheet1. Durées converties en minutes (1 h = 60 min).</t>
   </si>
 </sst>
 </file>
@@ -81,7 +81,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -153,8 +153,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -241,12 +249,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF7F7F7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF70AD47"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -270,7 +272,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="25">
+  <borders count="36">
     <border>
       <left/>
       <right/>
@@ -558,19 +560,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="hair">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="medium">
@@ -592,13 +581,157 @@
       <bottom style="medium">
         <color auto="1"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="hair">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color auto="1"/>
+      </left>
+      <right style="hair">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -636,8 +769,6 @@
     <xf numFmtId="164" fontId="0" fillId="14" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -662,11 +793,9 @@
     <xf numFmtId="1" fontId="0" fillId="14" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="13" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -680,18 +809,8 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="18" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="17" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="12" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -700,23 +819,87 @@
     <xf numFmtId="1" fontId="0" fillId="14" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="1" fillId="17" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="19" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="17" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="19" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="17" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="19" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="1" fontId="1" fillId="18" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="18" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="18" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="11" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="16" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="16" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="11" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="16" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="30" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="14" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="14" borderId="21" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="14" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="12" borderId="31" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="12" borderId="32" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="12" borderId="32" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="33" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="14" borderId="31" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="14" borderId="32" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="14" borderId="32" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="33" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="35" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1033,9 +1216,6 @@
   <wetp:taskpane dockstate="right" visibility="0" width="438" row="1">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
-  <wetp:taskpane dockstate="right" visibility="0" width="438" row="1">
-    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-  </wetp:taskpane>
 </wetp:taskpanes>
 </file>
 
@@ -1053,38 +1233,24 @@
 </we:webextension>
 </file>
 
-<file path=xl/webextensions/webextension2.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{3ADA3ED5-DD28-4B9A-BDB0-6749AF8E7D97}">
-  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
-  <we:alternateReferences>
-    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
-  </we:alternateReferences>
-  <we:properties>
-    <we:property name="claude.fileId" value="&quot;db861573-e0e8-43be-b027-a3e279b75f8c&quot;"/>
-  </we:properties>
-  <we:bindings/>
-  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</we:webextension>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9E6E333-5EC4-488E-9B0A-5C5E52B64EBC}">
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:10" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
-      <c r="I1" s="49"/>
-      <c r="J1" s="49"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
     </row>
     <row r="2" spans="1:10" ht="4.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
@@ -1099,42 +1265,42 @@
       <c r="J2" s="1"/>
     </row>
     <row r="3" spans="1:10" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="69" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="50" t="s">
+      <c r="B3" s="62" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="50"/>
-      <c r="D3" s="51"/>
-      <c r="E3" s="52"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="64"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="53" t="s">
+      <c r="G3" s="65" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="54"/>
-      <c r="I3" s="55"/>
-      <c r="J3" s="56"/>
+      <c r="H3" s="66"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="68"/>
     </row>
     <row r="4" spans="1:10" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="58"/>
+      <c r="A4" s="70"/>
       <c r="B4" s="4" t="s">
         <v>0</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="20" t="s">
+      <c r="E4" s="18" t="s">
         <v>8</v>
       </c>
       <c r="F4" s="3"/>
-      <c r="G4" s="26" t="s">
+      <c r="G4" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="H4" s="22" t="s">
+      <c r="H4" s="20" t="s">
         <v>6</v>
       </c>
       <c r="I4" s="5" t="s">
@@ -1154,17 +1320,17 @@
       <c r="C5" s="8">
         <v>1019</v>
       </c>
-      <c r="D5" s="18">
+      <c r="D5" s="16">
         <v>46.68</v>
       </c>
-      <c r="E5" s="21">
+      <c r="E5" s="19">
         <v>0.92200000000000004</v>
       </c>
       <c r="F5" s="3"/>
-      <c r="G5" s="41">
+      <c r="G5" s="31">
         <v>25110705</v>
       </c>
-      <c r="H5" s="23">
+      <c r="H5" s="21">
         <v>737</v>
       </c>
       <c r="I5" s="9">
@@ -1184,17 +1350,17 @@
       <c r="C6" s="12">
         <v>725</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="17" t="s">
         <v>1</v>
       </c>
       <c r="E6" s="14">
         <v>0.81799999999999995</v>
       </c>
       <c r="F6" s="3"/>
-      <c r="G6" s="42">
+      <c r="G6" s="32">
         <v>25480433</v>
       </c>
-      <c r="H6" s="24">
+      <c r="H6" s="22">
         <v>885</v>
       </c>
       <c r="I6" s="13">
@@ -1214,17 +1380,17 @@
       <c r="C7" s="8">
         <v>668</v>
       </c>
-      <c r="D7" s="18">
+      <c r="D7" s="16">
         <v>42</v>
       </c>
-      <c r="E7" s="21">
+      <c r="E7" s="19">
         <v>0.82399999999999995</v>
       </c>
       <c r="F7" s="3"/>
-      <c r="G7" s="41">
+      <c r="G7" s="31">
         <v>25500396</v>
       </c>
-      <c r="H7" s="23">
+      <c r="H7" s="21">
         <v>841</v>
       </c>
       <c r="I7" s="9">
@@ -1244,17 +1410,17 @@
       <c r="C8" s="12">
         <v>1114</v>
       </c>
-      <c r="D8" s="19">
+      <c r="D8" s="17">
         <v>47.82</v>
       </c>
       <c r="E8" s="14">
         <v>0.72</v>
       </c>
       <c r="F8" s="3"/>
-      <c r="G8" s="42">
+      <c r="G8" s="32">
         <v>26030732</v>
       </c>
-      <c r="H8" s="24">
+      <c r="H8" s="22">
         <v>893</v>
       </c>
       <c r="I8" s="13">
@@ -1274,17 +1440,17 @@
       <c r="C9" s="8">
         <v>923</v>
       </c>
-      <c r="D9" s="18">
+      <c r="D9" s="16">
         <v>48.91</v>
       </c>
-      <c r="E9" s="21">
+      <c r="E9" s="19">
         <v>1.1399999999999999</v>
       </c>
       <c r="F9" s="3"/>
-      <c r="G9" s="41">
+      <c r="G9" s="31">
         <v>26040641</v>
       </c>
-      <c r="H9" s="23">
+      <c r="H9" s="21">
         <v>745</v>
       </c>
       <c r="I9" s="9">
@@ -1304,17 +1470,17 @@
       <c r="C10" s="12">
         <v>775</v>
       </c>
-      <c r="D10" s="19">
+      <c r="D10" s="17">
         <v>43.2</v>
       </c>
       <c r="E10" s="14">
         <v>0.92</v>
       </c>
       <c r="F10" s="3"/>
-      <c r="G10" s="42">
+      <c r="G10" s="32">
         <v>26040642</v>
       </c>
-      <c r="H10" s="24">
+      <c r="H10" s="22">
         <v>669</v>
       </c>
       <c r="I10" s="13" t="s">
@@ -1334,17 +1500,17 @@
       <c r="C11" s="8">
         <v>1472</v>
       </c>
-      <c r="D11" s="18">
+      <c r="D11" s="16">
         <v>49.69</v>
       </c>
-      <c r="E11" s="21">
+      <c r="E11" s="19">
         <v>1.2110000000000001</v>
       </c>
       <c r="F11" s="3"/>
-      <c r="G11" s="41">
+      <c r="G11" s="31">
         <v>26160265</v>
       </c>
-      <c r="H11" s="23">
+      <c r="H11" s="21">
         <v>771</v>
       </c>
       <c r="I11" s="9">
@@ -1364,23 +1530,23 @@
       <c r="C12" s="12">
         <v>939</v>
       </c>
-      <c r="D12" s="19">
+      <c r="D12" s="17">
         <v>49.54</v>
       </c>
       <c r="E12" s="14">
         <v>1.109</v>
       </c>
       <c r="F12" s="3"/>
-      <c r="G12" s="42">
+      <c r="G12" s="46">
         <v>25140526</v>
       </c>
-      <c r="H12" s="24">
+      <c r="H12" s="47">
         <v>912</v>
       </c>
-      <c r="I12" s="13">
+      <c r="I12" s="48">
         <v>49.81</v>
       </c>
-      <c r="J12" s="14">
+      <c r="J12" s="27">
         <v>0.92500000000000004</v>
       </c>
     </row>
@@ -1394,17 +1560,25 @@
       <c r="C13" s="8">
         <v>755</v>
       </c>
-      <c r="D13" s="18">
+      <c r="D13" s="16">
         <v>49.49</v>
       </c>
-      <c r="E13" s="21">
+      <c r="E13" s="19">
         <v>0.747</v>
       </c>
       <c r="F13" s="3"/>
-      <c r="G13" s="27"/>
-      <c r="H13" s="25"/>
-      <c r="I13" s="15"/>
-      <c r="J13" s="16"/>
+      <c r="G13" s="49">
+        <v>25050369</v>
+      </c>
+      <c r="H13" s="50">
+        <v>760.2</v>
+      </c>
+      <c r="I13" s="51">
+        <v>45.01</v>
+      </c>
+      <c r="J13" s="52">
+        <v>0.78900000000000003</v>
+      </c>
     </row>
     <row r="14" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11">
@@ -1416,17 +1590,25 @@
       <c r="C14" s="12">
         <v>778</v>
       </c>
-      <c r="D14" s="19">
+      <c r="D14" s="17">
         <v>48.82</v>
       </c>
       <c r="E14" s="14">
         <v>0.71399999999999997</v>
       </c>
       <c r="F14" s="3"/>
-      <c r="G14" s="27"/>
-      <c r="H14" s="25"/>
-      <c r="I14" s="15"/>
-      <c r="J14" s="16"/>
+      <c r="G14" s="53">
+        <v>26030731</v>
+      </c>
+      <c r="H14" s="54">
+        <v>1185</v>
+      </c>
+      <c r="I14" s="55">
+        <v>49.84</v>
+      </c>
+      <c r="J14" s="56">
+        <v>0.82099999999999995</v>
+      </c>
     </row>
     <row r="15" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="7">
@@ -1438,17 +1620,25 @@
       <c r="C15" s="8">
         <v>560</v>
       </c>
-      <c r="D15" s="18">
+      <c r="D15" s="16">
         <v>49.3</v>
       </c>
-      <c r="E15" s="21">
+      <c r="E15" s="19">
         <v>0.76</v>
       </c>
       <c r="F15" s="3"/>
-      <c r="G15" s="27"/>
-      <c r="H15" s="25"/>
-      <c r="I15" s="15"/>
-      <c r="J15" s="16"/>
+      <c r="G15" s="49">
+        <v>26020521</v>
+      </c>
+      <c r="H15" s="50">
+        <v>679.8</v>
+      </c>
+      <c r="I15" s="51">
+        <v>54.25</v>
+      </c>
+      <c r="J15" s="52">
+        <v>0.72899999999999998</v>
+      </c>
     </row>
     <row r="16" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="11">
@@ -1460,17 +1650,25 @@
       <c r="C16" s="12">
         <v>641</v>
       </c>
-      <c r="D16" s="19">
+      <c r="D16" s="17">
         <v>47.67</v>
       </c>
       <c r="E16" s="14">
         <v>0.82499999999999996</v>
       </c>
       <c r="F16" s="3"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="25"/>
-      <c r="I16" s="15"/>
-      <c r="J16" s="16"/>
+      <c r="G16" s="53">
+        <v>26020519</v>
+      </c>
+      <c r="H16" s="54">
+        <v>1200</v>
+      </c>
+      <c r="I16" s="55">
+        <v>52.46</v>
+      </c>
+      <c r="J16" s="56">
+        <v>0.74299999999999999</v>
+      </c>
     </row>
     <row r="17" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7">
@@ -1482,221 +1680,270 @@
       <c r="C17" s="8">
         <v>751</v>
       </c>
-      <c r="D17" s="18">
+      <c r="D17" s="16">
         <v>49.12</v>
       </c>
-      <c r="E17" s="21">
+      <c r="E17" s="19">
         <v>0.61299999999999999</v>
       </c>
       <c r="F17" s="3"/>
-      <c r="G17" s="27"/>
-      <c r="H17" s="25"/>
-      <c r="I17" s="15"/>
-      <c r="J17" s="16"/>
+      <c r="G17" s="31"/>
+      <c r="H17" s="21"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="10"/>
     </row>
     <row r="18" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="11">
         <v>14</v>
       </c>
       <c r="B18" s="12">
-        <v>25140527</v>
+        <v>25200590</v>
       </c>
       <c r="C18" s="12">
-        <v>751</v>
-      </c>
-      <c r="D18" s="19">
-        <v>49.12</v>
+        <v>1054</v>
+      </c>
+      <c r="D18" s="17">
+        <v>42.77</v>
       </c>
       <c r="E18" s="14">
-        <v>0.61299999999999999</v>
+        <v>0.77200000000000002</v>
       </c>
       <c r="F18" s="3"/>
-      <c r="G18" s="27"/>
-      <c r="H18" s="25"/>
-      <c r="I18" s="15"/>
-      <c r="J18" s="16"/>
+      <c r="G18" s="32"/>
+      <c r="H18" s="22"/>
+      <c r="I18" s="13"/>
+      <c r="J18" s="14"/>
     </row>
     <row r="19" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="7">
         <v>15</v>
       </c>
       <c r="B19" s="8">
-        <v>25200590</v>
+        <v>26020520</v>
       </c>
       <c r="C19" s="8">
-        <v>1054</v>
-      </c>
-      <c r="D19" s="18">
-        <v>42.77</v>
-      </c>
-      <c r="E19" s="21">
-        <v>0.77200000000000002</v>
+        <v>741</v>
+      </c>
+      <c r="D19" s="16">
+        <v>58.86</v>
+      </c>
+      <c r="E19" s="19">
+        <v>0.57499999999999996</v>
       </c>
       <c r="F19" s="3"/>
-      <c r="G19" s="27"/>
-      <c r="H19" s="25"/>
-      <c r="I19" s="15"/>
-      <c r="J19" s="16"/>
+      <c r="G19" s="31"/>
+      <c r="H19" s="21"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="10"/>
     </row>
     <row r="20" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="11">
         <v>16</v>
       </c>
       <c r="B20" s="12">
-        <v>26020520</v>
+        <v>26040643</v>
       </c>
       <c r="C20" s="12">
-        <v>741</v>
-      </c>
-      <c r="D20" s="19">
-        <v>58.86</v>
+        <v>715</v>
+      </c>
+      <c r="D20" s="17">
+        <v>48.52</v>
       </c>
       <c r="E20" s="14">
-        <v>0.57499999999999996</v>
+        <v>1.321</v>
       </c>
       <c r="F20" s="3"/>
-      <c r="G20" s="27"/>
-      <c r="H20" s="25"/>
-      <c r="I20" s="15"/>
-      <c r="J20" s="16"/>
+      <c r="G20" s="31"/>
+      <c r="H20" s="21"/>
+      <c r="I20" s="9"/>
+      <c r="J20" s="10"/>
     </row>
     <row r="21" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="7">
         <v>17</v>
       </c>
       <c r="B21" s="8">
-        <v>26040643</v>
+        <v>26130338</v>
       </c>
       <c r="C21" s="8">
-        <v>715</v>
-      </c>
-      <c r="D21" s="18">
-        <v>48.52</v>
-      </c>
-      <c r="E21" s="21">
-        <v>1.321</v>
+        <v>721</v>
+      </c>
+      <c r="D21" s="16">
+        <v>49.75</v>
+      </c>
+      <c r="E21" s="19">
+        <v>1.171</v>
       </c>
       <c r="F21" s="3"/>
-      <c r="G21" s="27"/>
-      <c r="H21" s="25"/>
-      <c r="I21" s="15"/>
-      <c r="J21" s="16"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="22"/>
+      <c r="I21" s="13"/>
+      <c r="J21" s="14"/>
     </row>
     <row r="22" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="11">
         <v>18</v>
       </c>
       <c r="B22" s="12">
-        <v>26130338</v>
+        <v>26160263</v>
       </c>
       <c r="C22" s="12">
-        <v>721</v>
-      </c>
-      <c r="D22" s="19">
-        <v>49.75</v>
+        <v>1022</v>
+      </c>
+      <c r="D22" s="17">
+        <v>46.98</v>
       </c>
       <c r="E22" s="14">
-        <v>1.171</v>
+        <v>0.73399999999999999</v>
       </c>
       <c r="F22" s="3"/>
-      <c r="G22" s="27"/>
-      <c r="H22" s="25"/>
-      <c r="I22" s="15"/>
-      <c r="J22" s="16"/>
+      <c r="G22" s="31"/>
+      <c r="H22" s="21"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="10"/>
     </row>
     <row r="23" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="7">
         <v>19</v>
       </c>
       <c r="B23" s="8">
-        <v>26160263</v>
+        <v>26160264</v>
       </c>
       <c r="C23" s="8">
-        <v>1022</v>
-      </c>
-      <c r="D23" s="18">
-        <v>46.98</v>
-      </c>
-      <c r="E23" s="21">
-        <v>0.73399999999999999</v>
+        <v>873</v>
+      </c>
+      <c r="D23" s="16">
+        <v>48.84</v>
+      </c>
+      <c r="E23" s="19">
+        <v>0.94199999999999995</v>
       </c>
       <c r="F23" s="3"/>
-      <c r="G23" s="27"/>
-      <c r="H23" s="25"/>
-      <c r="I23" s="15"/>
-      <c r="J23" s="16"/>
-    </row>
-    <row r="24" spans="1:10" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="28">
+      <c r="G23" s="31"/>
+      <c r="H23" s="21"/>
+      <c r="I23" s="9"/>
+      <c r="J23" s="10"/>
+    </row>
+    <row r="24" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="24">
         <v>20</v>
       </c>
-      <c r="B24" s="29">
-        <v>26160264</v>
-      </c>
-      <c r="C24" s="29">
-        <v>873</v>
-      </c>
-      <c r="D24" s="30">
-        <v>48.84</v>
-      </c>
-      <c r="E24" s="31">
-        <v>0.94199999999999995</v>
-      </c>
-      <c r="F24" s="32"/>
-      <c r="G24" s="33"/>
-      <c r="H24" s="34"/>
-      <c r="I24" s="35"/>
-      <c r="J24" s="36"/>
-    </row>
-    <row r="25" spans="1:10" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="37" t="s">
+      <c r="B24" s="25">
+        <v>25190285</v>
+      </c>
+      <c r="C24" s="25">
+        <v>1024.8</v>
+      </c>
+      <c r="D24" s="26">
+        <v>44.67</v>
+      </c>
+      <c r="E24" s="27">
+        <v>0.92800000000000005</v>
+      </c>
+      <c r="F24" s="28"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="22"/>
+      <c r="I24" s="13"/>
+      <c r="J24" s="14"/>
+    </row>
+    <row r="25" spans="1:10" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="57">
+        <v>21</v>
+      </c>
+      <c r="B25" s="58">
+        <v>25020345</v>
+      </c>
+      <c r="C25" s="58">
+        <f>11.83*60</f>
+        <v>709.8</v>
+      </c>
+      <c r="D25" s="59">
+        <v>43.94</v>
+      </c>
+      <c r="E25" s="60">
+        <v>0.83299999999999996</v>
+      </c>
+      <c r="F25" s="36"/>
+      <c r="G25" s="31"/>
+      <c r="H25" s="21"/>
+      <c r="I25" s="9"/>
+      <c r="J25" s="10"/>
+    </row>
+    <row r="26" spans="1:10" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="38">
+        <v>22</v>
+      </c>
+      <c r="B26" s="40">
+        <f>25190285</f>
+        <v>25190285</v>
+      </c>
+      <c r="C26" s="40">
+        <f>1025</f>
+        <v>1025</v>
+      </c>
+      <c r="D26" s="43">
+        <f>44.67</f>
+        <v>44.67</v>
+      </c>
+      <c r="E26" s="45">
+        <f>0.928</f>
+        <v>0.92800000000000005</v>
+      </c>
+      <c r="F26" s="36"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="21"/>
+      <c r="I26" s="9"/>
+      <c r="J26" s="10"/>
+    </row>
+    <row r="27" spans="1:10" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="37" t="s">
         <v>9</v>
       </c>
-      <c r="B25" s="38" t="s">
+      <c r="B27" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="C25" s="43">
-        <f>AVERAGE(C5:C24)</f>
-        <v>849.85</v>
-      </c>
-      <c r="D25" s="45">
-        <f>AVERAGE(D5:D24)</f>
-        <v>48.26736842105263</v>
-      </c>
-      <c r="E25" s="47">
-        <f>AVERAGE(E5:E24)</f>
-        <v>0.87254999999999983</v>
-      </c>
-      <c r="F25" s="39"/>
-      <c r="G25" s="40" t="s">
+      <c r="C27" s="41">
+        <f>AVERAGE(C5:C26)</f>
+        <v>863.89090909090908</v>
+      </c>
+      <c r="D27" s="42">
+        <f>AVERAGE(D5:D26)</f>
+        <v>47.678095238095231</v>
+      </c>
+      <c r="E27" s="44">
+        <f>AVERAGE(E5:E26)</f>
+        <v>0.88759090909090899</v>
+      </c>
+      <c r="F27" s="29"/>
+      <c r="G27" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="H25" s="44">
-        <f>AVERAGE(H5:H12)</f>
-        <v>806.625</v>
-      </c>
-      <c r="I25" s="46">
-        <f>AVERAGE(I5:I12)</f>
-        <v>50.135714285714286</v>
-      </c>
-      <c r="J25" s="48">
-        <f>AVERAGE(J5:J12)</f>
-        <v>0.98062499999999986</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="59" t="s">
+      <c r="H27" s="33">
+        <f>AVERAGE(H5:H16)</f>
+        <v>856.5</v>
+      </c>
+      <c r="I27" s="34">
+        <f>AVERAGE(I5:I16)</f>
+        <v>50.228181818181817</v>
+      </c>
+      <c r="J27" s="35">
+        <f>AVERAGE(J5:J16)</f>
+        <v>0.91058333333333319</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="71" t="s">
         <v>11</v>
       </c>
-      <c r="B27" s="60"/>
-      <c r="C27" s="60"/>
-      <c r="D27" s="60"/>
-      <c r="E27" s="60"/>
-      <c r="F27" s="60"/>
-      <c r="G27" s="60"/>
-      <c r="H27" s="60"/>
-      <c r="I27" s="60"/>
-      <c r="J27" s="60"/>
+      <c r="B29" s="72"/>
+      <c r="C29" s="72"/>
+      <c r="D29" s="72"/>
+      <c r="E29" s="72"/>
+      <c r="F29" s="72"/>
+      <c r="G29" s="72"/>
+      <c r="H29" s="72"/>
+      <c r="I29" s="72"/>
+      <c r="J29" s="72"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1704,7 +1951,7 @@
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="G3:J3"/>
     <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A27:J27"/>
+    <mergeCell ref="A29:J29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>